<commit_message>
updating tracking. Shifting estimates to sat morning as in theory that should be end of the week i.e. a full weeks workout done. making some adjustments to layout
</commit_message>
<xml_diff>
--- a/Tracking.xlsx
+++ b/Tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\c.campbell\source\LearningResourcesRepo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25292D07-4F85-4BC1-92DD-2932D324B9C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B10A3AF6-69EE-4A4B-AA73-1E5EDE48C03B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="39">
   <si>
     <t>Week Start</t>
   </si>
@@ -153,6 +153,12 @@
   </si>
   <si>
     <t>**Dehydration weight lol</t>
+  </si>
+  <si>
+    <t>1st april</t>
+  </si>
+  <si>
+    <t>7th april</t>
   </si>
 </sst>
 </file>
@@ -194,7 +200,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -222,6 +228,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.34998626667073579"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -267,7 +279,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -327,14 +339,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1107,11 +1142,13 @@
       <c r="D5" s="5">
         <v>144</v>
       </c>
-      <c r="E5" s="1"/>
-      <c r="F5" s="21">
+      <c r="E5" s="1">
+        <v>143.80000000000001</v>
+      </c>
+      <c r="F5" s="21"/>
+      <c r="G5" s="28">
         <v>144.1</v>
       </c>
-      <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" t="s">
         <v>36</v>
@@ -1125,10 +1162,10 @@
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
-      <c r="F6" s="21">
+      <c r="F6" s="21"/>
+      <c r="G6" s="28">
         <v>142.9</v>
       </c>
-      <c r="G6" s="1"/>
       <c r="H6" s="1"/>
     </row>
     <row r="7" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1136,14 +1173,12 @@
         <v>20</v>
       </c>
       <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="22">
-        <v>141.4</v>
-      </c>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="26"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="25"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1153,7 +1188,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D74EBFC-9222-4BC1-BD99-1A369ED9D387}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.44140625" customWidth="1"/>
@@ -1162,6 +1197,7 @@
     <col min="4" max="4" width="24.6640625" customWidth="1"/>
     <col min="5" max="5" width="28" customWidth="1"/>
     <col min="6" max="6" width="29" customWidth="1"/>
+    <col min="7" max="7" width="30.33203125" customWidth="1"/>
     <col min="8" max="8" width="29.77734375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1192,63 +1228,75 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="23">
-        <v>139.9</v>
-      </c>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
+      <c r="A2" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="24"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="29">
+        <v>141.4</v>
+      </c>
+      <c r="H2" s="22"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>22</v>
+      <c r="A3" s="13" t="s">
+        <v>38</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="21">
-        <v>138.4</v>
-      </c>
-      <c r="G3" s="1"/>
+      <c r="G3" s="30">
+        <v>139.9</v>
+      </c>
       <c r="H3" s="1"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
-      <c r="F4" s="21">
+      <c r="G4" s="28">
+        <v>138.4</v>
+      </c>
+      <c r="H4" s="1"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="G5" s="28">
         <v>136.9</v>
       </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-    </row>
-    <row r="5" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="17" t="s">
+      <c r="H5" s="1"/>
+    </row>
+    <row r="6" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="18"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="22">
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="31">
         <v>135.4</v>
       </c>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
+      <c r="H6" s="18"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1256,6 +1304,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F756905-7F71-46E7-A371-7B3817CD3583}">
   <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="7" max="7" width="22.88671875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="9" t="s">
@@ -1287,7 +1338,7 @@
       <c r="A2" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="21">
+      <c r="G2" s="28">
         <v>133.9</v>
       </c>
     </row>
@@ -1295,7 +1346,7 @@
       <c r="A3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="21">
+      <c r="G3" s="28">
         <v>132.4</v>
       </c>
     </row>
@@ -1303,7 +1354,7 @@
       <c r="A4" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="23">
+      <c r="G4" s="30">
         <v>130.9</v>
       </c>
     </row>
@@ -1315,10 +1366,10 @@
       <c r="C5" s="18"/>
       <c r="D5" s="18"/>
       <c r="E5" s="18"/>
-      <c r="F5" s="22">
+      <c r="F5" s="18"/>
+      <c r="G5" s="31">
         <v>129.4</v>
       </c>
-      <c r="G5" s="18"/>
       <c r="H5" s="18"/>
     </row>
   </sheetData>
@@ -1330,6 +1381,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEEB2055-4920-46DD-81EA-82AFF7E2861B}">
   <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="7" max="7" width="15.44140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="9" t="s">
@@ -1361,7 +1415,7 @@
       <c r="A2" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="F2" s="21">
+      <c r="G2" s="28">
         <v>127.9</v>
       </c>
     </row>
@@ -1369,7 +1423,7 @@
       <c r="A3" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="F3" s="21">
+      <c r="G3" s="28">
         <v>126.4</v>
       </c>
     </row>
@@ -1377,7 +1431,7 @@
       <c r="A4" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="F4" s="21">
+      <c r="G4" s="28">
         <v>124.9</v>
       </c>
     </row>
@@ -1385,7 +1439,7 @@
       <c r="A5" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F5" s="21">
+      <c r="G5" s="28">
         <v>123.4</v>
       </c>
     </row>
@@ -1397,10 +1451,10 @@
       <c r="C6" s="18"/>
       <c r="D6" s="18"/>
       <c r="E6" s="18"/>
-      <c r="F6" s="22">
+      <c r="F6" s="18"/>
+      <c r="G6" s="31">
         <v>121.9</v>
       </c>
-      <c r="G6" s="18"/>
       <c r="H6" s="18"/>
     </row>
   </sheetData>
@@ -1443,7 +1497,7 @@
       <c r="A2" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="F2" s="16">
+      <c r="F2" s="32">
         <v>120.4</v>
       </c>
     </row>

</xml_diff>